<commit_message>
Add 30 s vertical explainer video: German election system
- GermanElection composition (1080x1920, 30 fps, 900 frames): title, two
  votes, 5% threshold + 630-seat Bundestag, Chancellor majority (316),
  Federal Convention + President; persistent header, word-synced subtitles
- Offline Kokoro TTS voice-over and timeline generator; every animation,
  subtitle and sound effect is keyed off the generated timeline.json
- Synthesised royalty-free music bed (ducked under speech) and soft SFX
- render.sh renders and masters audio to -14 LUFS (npm run render:german-election)
- Script, storyboard, fact sheet and progress notes in briefs/german-election-system;
  brief spreadsheet example updated with the final script and timings

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BL29C7xRtjBshaeo3rcUPW
</commit_message>
<xml_diff>
--- a/briefs/motion-video-brief.xlsx
+++ b/briefs/motion-video-brief.xlsx
@@ -352,7 +352,7 @@
     <t xml:space="preserve">Words per second for a calm documentary voice (assumption, adjustable):</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: typical documentary narration is about 2.0-2.5 words/s (estimate by Claude)</t>
+    <t xml:space="preserve">Measured on the German election video: the voice reads about 2.3 spoken words/s, but numbers like 630 are spoken as 4 words and pauses between sentences take time - so plan at most about 2.1 on-screen words per second of scene time.</t>
   </si>
   <si>
     <t xml:space="preserve">Scene</t>
@@ -385,7 +385,7 @@
     <t xml:space="preserve">1 Title</t>
   </si>
   <si>
-    <t xml:space="preserve">Black background, German-flag stripes slide in; title 'German election system'</t>
+    <t xml:space="preserve">Germany map fills with black-red-gold stripes; Berlin pin; title 'German election system'</t>
   </si>
   <si>
     <t xml:space="preserve">How does Germany choose its leaders?</t>
@@ -394,7 +394,7 @@
     <t xml:space="preserve">2 Two votes</t>
   </si>
   <si>
-    <t xml:space="preserve">Ballot icon splits into two: person icon (1st vote) and party icon (2nd vote)</t>
+    <t xml:space="preserve">Ballot with two columns; crosses drawn; arrows to 'Local candidate' and 'Party strength' cards</t>
   </si>
   <si>
     <t xml:space="preserve">Voters cast two votes. The first picks a local candidate. The second decides each party's strength.</t>
@@ -403,34 +403,34 @@
     <t xml:space="preserve">3 Bundestag</t>
   </si>
   <si>
-    <t xml:space="preserve">5% bar chart threshold, then a parliament arc fills with 630 dots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parties need five percent to enter. Together, 630 members make up the Bundestag.</t>
+    <t xml:space="preserve">Bar chart with a dashed 5% line; then a 630-seat hemicycle builds with a counter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parties need 5% to enter. The Bundestag has 630 seats.</t>
   </si>
   <si>
     <t xml:space="preserve">4 Chancellor</t>
   </si>
   <si>
-    <t xml:space="preserve">Parliament arc points to a Chancellor icon; counter reaches 316 votes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Bundestag elects the Chancellor, with at least 316 votes. Today, that is Friedrich Merz.</t>
+    <t xml:space="preserve">316 seats turn gold (majority); Chancellor name card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It elects the Chancellor, with at least 316 votes. Today: Friedrich Merz.</t>
   </si>
   <si>
     <t xml:space="preserve">5 President</t>
   </si>
   <si>
-    <t xml:space="preserve">Separate Federal Convention circle points to a President icon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The President is chosen separately, by a Federal Convention. Today: Frank-Walter Steinmeier.</t>
+    <t xml:space="preserve">Hemicycle + 630 state delegates form the Federal Convention ring around the President; name card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The President is chosen by a Federal Convention. Today: Frank-Walter Steinmeier.</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: yellow cells are editable. Facts (630 seats, 316 majority, Merz, Steinmeier) are checked on 2026-10-13; Steinmeier's term ends in 2027 - re-check before publishing.</t>
+    <t xml:space="preserve">Notes: yellow cells are editable. This sheet shows the FINAL script and scene lengths of the German election video (timings come from the generated voice-over; details in briefs/german-election-system/). Facts (630 seats, 316 majority, Merz, Steinmeier) checked on 2026-10-13; Steinmeier's term ends 18 March 2027 - re-check before publishing.</t>
   </si>
 </sst>
 </file>
@@ -569,20 +569,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -602,7 +606,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -614,7 +618,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -873,67 +877,67 @@
   <dimension ref="A1:A13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="95"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -956,337 +960,337 @@
   <dimension ref="A1:D31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="C2" s="8"/>
+      <c r="D2" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
-      <c r="B3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6"/>
+      <c r="B3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="8"/>
+      <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="6" t="s">
+      <c r="C7" s="8"/>
+      <c r="D7" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="6" t="s">
+      <c r="C8" s="8"/>
+      <c r="D8" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6"/>
+      <c r="B9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="6" t="s">
+      <c r="C9" s="8"/>
+      <c r="D9" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6"/>
+      <c r="B10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="6" t="s">
+      <c r="C10" s="8"/>
+      <c r="D10" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="6" t="s">
+      <c r="C11" s="8"/>
+      <c r="D11" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6"/>
+      <c r="B12" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="6" t="s">
+      <c r="C12" s="8"/>
+      <c r="D12" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6"/>
+      <c r="B13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="6" t="s">
+      <c r="C13" s="8"/>
+      <c r="D13" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6"/>
+      <c r="B14" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="6" t="s">
+      <c r="C14" s="8"/>
+      <c r="D14" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="6" t="s">
+      <c r="C15" s="8"/>
+      <c r="D15" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="6" t="s">
+      <c r="C16" s="8"/>
+      <c r="D16" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="6" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6"/>
+      <c r="B17" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="6" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="6" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6"/>
+      <c r="B18" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="6" t="s">
+      <c r="C18" s="8"/>
+      <c r="D18" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6"/>
+      <c r="B19" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="6" t="s">
+      <c r="C19" s="8"/>
+      <c r="D19" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="6" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6"/>
+      <c r="B20" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="6" t="s">
+      <c r="C20" s="8"/>
+      <c r="D20" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="6" t="s">
+      <c r="C21" s="8"/>
+      <c r="D21" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6"/>
+      <c r="B22" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="6" t="s">
+      <c r="C22" s="8"/>
+      <c r="D22" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6"/>
+      <c r="B23" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="6" t="s">
+      <c r="C23" s="8"/>
+      <c r="D23" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6"/>
+      <c r="B24" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="6" t="s">
+      <c r="C24" s="8"/>
+      <c r="D24" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="6" t="s">
+      <c r="C25" s="8"/>
+      <c r="D25" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6"/>
+      <c r="B26" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="6" t="s">
+      <c r="C26" s="8"/>
+      <c r="D26" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="6" t="s">
+      <c r="C27" s="8"/>
+      <c r="D27" s="7" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6"/>
+      <c r="B28" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="6" t="s">
+      <c r="C28" s="8"/>
+      <c r="D28" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="6" t="s">
+      <c r="C29" s="8"/>
+      <c r="D29" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5"/>
-      <c r="B30" s="6" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6"/>
+      <c r="B30" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="6" t="s">
+      <c r="C30" s="8"/>
+      <c r="D30" s="7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="6" t="s">
+      <c r="C31" s="8"/>
+      <c r="D31" s="7" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1309,397 +1313,397 @@
   <dimension ref="A1:D31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
-      <c r="B3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6"/>
+      <c r="B3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6" t="s">
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6"/>
+      <c r="B9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6"/>
+      <c r="B10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6"/>
+      <c r="B12" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6"/>
+      <c r="B13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6"/>
+      <c r="B14" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="6" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6"/>
+      <c r="B17" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="6" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6"/>
+      <c r="B18" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6"/>
+      <c r="B19" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="6" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6"/>
+      <c r="B20" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6"/>
+      <c r="B22" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6"/>
+      <c r="B23" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6"/>
+      <c r="B24" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6"/>
+      <c r="B26" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="7" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6"/>
+      <c r="B28" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5"/>
-      <c r="B30" s="6" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6"/>
+      <c r="B30" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="7" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1722,250 +1726,250 @@
   <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="8" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="F1" s="9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
+    <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="10" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" s="6" t="n">
+      <c r="C4" s="8" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D4" s="7" t="n">
         <f aca="false">B4+C4</f>
-        <v>4</v>
-      </c>
-      <c r="E4" s="7" t="s">
+        <v>3.1</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="7" t="n">
         <f aca="false">LEN(TRIM(F4))-LEN(SUBSTITUTE(TRIM(F4)," ",""))+1</f>
         <v>6</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="11" t="n">
         <f aca="false">IF(C4=0,0,G4/C4)</f>
-        <v>1.5</v>
-      </c>
-      <c r="I4" s="6" t="str">
+        <v>1.93548387096774</v>
+      </c>
+      <c r="I4" s="7" t="str">
         <f aca="false">IF(H4&lt;=$F$1,"OK","Too fast")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <f aca="false">D4</f>
-        <v>4</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D5" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="D5" s="7" t="n">
         <f aca="false">B5+C5</f>
-        <v>11</v>
-      </c>
-      <c r="E5" s="7" t="s">
+        <v>10.8</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <f aca="false">LEN(TRIM(F5))-LEN(SUBSTITUTE(TRIM(F5)," ",""))+1</f>
         <v>16</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="11" t="n">
         <f aca="false">IF(C5=0,0,G5/C5)</f>
-        <v>2.28571428571429</v>
-      </c>
-      <c r="I5" s="6" t="str">
+        <v>2.07792207792208</v>
+      </c>
+      <c r="I5" s="7" t="str">
         <f aca="false">IF(H5&lt;=$F$1,"OK","Too fast")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <f aca="false">D5</f>
-        <v>11</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" s="6" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D6" s="7" t="n">
         <f aca="false">B6+C6</f>
-        <v>17</v>
-      </c>
-      <c r="E6" s="7" t="s">
+        <v>17.1</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <f aca="false">LEN(TRIM(F6))-LEN(SUBSTITUTE(TRIM(F6)," ",""))+1</f>
-        <v>13</v>
-      </c>
-      <c r="H6" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" s="11" t="n">
         <f aca="false">IF(C6=0,0,G6/C6)</f>
-        <v>2.16666666666667</v>
-      </c>
-      <c r="I6" s="6" t="str">
+        <v>1.58730158730159</v>
+      </c>
+      <c r="I6" s="7" t="str">
         <f aca="false">IF(H6&lt;=$F$1,"OK","Too fast")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <f aca="false">D6</f>
-        <v>17</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D7" s="6" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D7" s="7" t="n">
         <f aca="false">B7+C7</f>
-        <v>24</v>
-      </c>
-      <c r="E7" s="7" t="s">
+        <v>23.4</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="7" t="n">
         <f aca="false">LEN(TRIM(F7))-LEN(SUBSTITUTE(TRIM(F7)," ",""))+1</f>
-        <v>15</v>
-      </c>
-      <c r="H7" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H7" s="11" t="n">
         <f aca="false">IF(C7=0,0,G7/C7)</f>
-        <v>2.14285714285714</v>
-      </c>
-      <c r="I7" s="6" t="str">
+        <v>1.9047619047619</v>
+      </c>
+      <c r="I7" s="7" t="str">
         <f aca="false">IF(H7&lt;=$F$1,"OK","Too fast")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <f aca="false">D7</f>
-        <v>24</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="6" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D8" s="7" t="n">
         <f aca="false">B8+C8</f>
         <v>30</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="7" t="n">
         <f aca="false">LEN(TRIM(F8))-LEN(SUBSTITUTE(TRIM(F8)," ",""))+1</f>
-        <v>12</v>
-      </c>
-      <c r="H8" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H8" s="11" t="n">
         <f aca="false">IF(C8=0,0,G8/C8)</f>
-        <v>2</v>
-      </c>
-      <c r="I8" s="6" t="str">
+        <v>1.66666666666667</v>
+      </c>
+      <c r="I8" s="7" t="str">
         <f aca="false">IF(H8&lt;=$F$1,"OK","Too fast")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11" t="n">
+      <c r="B9" s="12"/>
+      <c r="C9" s="12" t="n">
         <f aca="false">SUM(C4:C8)</f>
         <v>30</v>
       </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11" t="n">
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12" t="n">
         <f aca="false">SUM(G4:G8)</f>
-        <v>62</v>
-      </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11" t="str">
-        <f aca="false">IF(C9=30,"30 s target met","Duration is "&amp;C9&amp;" s")</f>
+        <v>55</v>
+      </c>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12" t="str">
+        <f aca="false">IF(ROUND(C9,1)=30,"30 s target met","Duration is "&amp;ROUND(C9,1)&amp;" s")</f>
         <v>30 s target met</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>135</v>
       </c>
     </row>

</xml_diff>